<commit_message>
Updated Budget and Decisioni .xlsx files
</commit_message>
<xml_diff>
--- a/PULSE_Registro_Decisioni.xlsx
+++ b/PULSE_Registro_Decisioni.xlsx
@@ -4067,89 +4067,359 @@
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="26">
-      <c r="A44" s="47" t="n"/>
-      <c r="B44" s="48" t="n"/>
-      <c r="C44" s="47" t="n"/>
-      <c r="D44" s="47" t="n"/>
-      <c r="E44" s="47" t="n"/>
-      <c r="F44" s="47" t="n"/>
-      <c r="G44" s="47" t="n"/>
-      <c r="H44" s="47" t="n"/>
-      <c r="I44" s="47" t="n"/>
-      <c r="J44" s="47" t="n"/>
-      <c r="K44" s="47" t="n"/>
-      <c r="L44" s="47" t="n"/>
+      <c r="A44" s="47" t="inlineStr">
+        <is>
+          <t>D-043</t>
+        </is>
+      </c>
+      <c r="B44" s="48" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C44" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D44" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="E44" s="47" t="inlineStr">
+        <is>
+          <t>GNC</t>
+        </is>
+      </c>
+      <c r="F44" s="47" t="inlineStr">
+        <is>
+          <t>Orientamento di riferimento per il dimensionamento ADCS (L1): lato lungo (454 mm) verso nadir, telescopio che guarda lungo il lato lungo, faccia 226 × 454 mm sulla velocità (0,103 m²). Inerzie come inviluppo: trasversali (rollio, beccheggio) 0,64–1,14 kg·m², asse lungo (imbardata) 0,26–0,55 kg·m² (30 kg pieno → 36 kg guscio); massimo per coppia e momento delle ruote, minimo per la deriva; pannelli dispiegabili come sensibilità (~0,055 kg·m² per kg) fino ad A5.6</t>
+        </is>
+      </c>
+      <c r="G44" s="47" t="inlineStr">
+        <is>
+          <t>L2: lato lungo di traverso (telescopio in 226 mm, beccheggio sensibile ai disturbi); L3: lato lungo lungo la traccia (area 0,051 m², riapre A1-bis/D-022/D-033/D-034); valore unico d'inerzia</t>
+        </is>
+      </c>
+      <c r="H44" s="47" t="inlineStr">
+        <is>
+          <t>Coerente con l'area di drag di A1 (0,1 m²) e con ΔV e propulsione già decisi; focale 0,70 m ripiegabile lungo i 454 mm come l'imager 8U di EarthNext; gradiente di gravità stabilizzante a nadir. Inviluppo entro un fattore 1,8, coerente con la Fase A</t>
+        </is>
+      </c>
+      <c r="I44" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 c), d), e), g); layout del telescopio (Giuseppe); A5.7</t>
+        </is>
+      </c>
+      <c r="J44" s="47" t="inlineStr">
+        <is>
+          <t>DR-10, DR-11, DR-14</t>
+        </is>
+      </c>
+      <c r="K44" s="47" t="inlineStr">
+        <is>
+          <t>R-01, R-06</t>
+        </is>
+      </c>
+      <c r="L44" s="47" t="inlineStr">
+        <is>
+          <t>Proposta</t>
+        </is>
+      </c>
       <c r="M44" s="47" t="n"/>
-      <c r="N44" s="47" t="n"/>
-      <c r="O44" s="47" t="n"/>
+      <c r="N44" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 b) – chat del 24/10/2026</t>
+        </is>
+      </c>
+      <c r="O44" s="47" t="inlineStr">
+        <is>
+          <t>Proposta: fissa la posizione del telescopio di Giuseppe. TBC fino ad A5.7. DA VERIFICARE IN A5.7: REGULUS lunga 250 mm (V-01, valore prudente; altra tabella T4I 200 mm) contro 226,3 mm di involucro lungo X (direzione di spinta): controllare disegno T4I e posizione dell'ugello. Idea L3 (drag dimezzato) da rivalutare in A5.7 / Fase B</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="26">
-      <c r="A45" s="47" t="n"/>
-      <c r="B45" s="48" t="n"/>
-      <c r="C45" s="47" t="n"/>
-      <c r="D45" s="47" t="n"/>
-      <c r="E45" s="47" t="n"/>
-      <c r="F45" s="47" t="n"/>
-      <c r="G45" s="47" t="n"/>
-      <c r="H45" s="47" t="n"/>
-      <c r="I45" s="47" t="n"/>
-      <c r="J45" s="47" t="n"/>
-      <c r="K45" s="47" t="n"/>
-      <c r="L45" s="47" t="n"/>
+      <c r="A45" s="47" t="inlineStr">
+        <is>
+          <t>D-044</t>
+        </is>
+      </c>
+      <c r="B45" s="48" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C45" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D45" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="E45" s="47" t="inlineStr">
+        <is>
+          <t>GNC</t>
+        </is>
+      </c>
+      <c r="F45" s="47" t="inlineStr">
+        <is>
+          <t>Profilo nominale della FMC notturna: inseguimento continuo dal bordo della finestra (F2), aggancio alla linea di vista a 0,7–1,1°/s e scatti dove conviene; il colpo rapido (F1, rampa 2–9 s a 3–7·10⁻³ N·m) si simula come caso di stress</t>
+        </is>
+      </c>
+      <c r="G45" s="47" t="inlineStr">
+        <is>
+          <t>F1 come nominale; F3 aggancio anticipato di ~20–30 s</t>
+        </is>
+      </c>
+      <c r="H45" s="47" t="inlineStr">
+        <is>
+          <t>DR-10 chiede un moto dolce: con F2 la coppia richiesta è ~4,6·10⁻⁴ N·m (solo curvatura della LOS), decine di secondi per assestarsi, scatti mossi ripetibili nella finestra (47,7 s a 30°, 84 s a 45°). Momento max FMC 0,029 N·m·s (velocità inerziale 1,47°/s, I = 1,14 kg·m²)</t>
+        </is>
+      </c>
+      <c r="I45" s="47" t="inlineStr">
+        <is>
+          <t>Simulazione 1-asse (A5.3 c parte 2), giroscopio e star tracker ad alta velocità (A5.3 f), DR-11</t>
+        </is>
+      </c>
+      <c r="J45" s="47" t="inlineStr">
+        <is>
+          <t>DR-04, DR-08, DR-10, DR-11, DR-18</t>
+        </is>
+      </c>
+      <c r="K45" s="47" t="inlineStr">
+        <is>
+          <t>R-06, R-21, R-25</t>
+        </is>
+      </c>
+      <c r="L45" s="47" t="inlineStr">
+        <is>
+          <t>Approvata</t>
+        </is>
+      </c>
       <c r="M45" s="47" t="n"/>
-      <c r="N45" s="47" t="n"/>
-      <c r="O45" s="47" t="n"/>
+      <c r="N45" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 c) – chat del 24/10/2026</t>
+        </is>
+      </c>
+      <c r="O45" s="47" t="inlineStr">
+        <is>
+          <t>Riguarda solo la parte GNC: non cambia numeri di Giuseppe (10–15 scatti da 20 ms invariati). Costo: assetto a 1–1,5°/s per tutta la finestra, conoscenza affidata al giroscopio</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="26">
-      <c r="A46" s="47" t="n"/>
-      <c r="B46" s="48" t="n"/>
-      <c r="C46" s="47" t="n"/>
-      <c r="D46" s="47" t="n"/>
-      <c r="E46" s="47" t="n"/>
-      <c r="F46" s="47" t="n"/>
-      <c r="G46" s="47" t="n"/>
-      <c r="H46" s="47" t="n"/>
-      <c r="I46" s="47" t="n"/>
-      <c r="J46" s="47" t="n"/>
-      <c r="K46" s="47" t="n"/>
-      <c r="L46" s="47" t="n"/>
+      <c r="A46" s="47" t="inlineStr">
+        <is>
+          <t>D-045</t>
+        </is>
+      </c>
+      <c r="B46" s="48" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C46" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D46" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="E46" s="47" t="inlineStr">
+        <is>
+          <t>GNC</t>
+        </is>
+      </c>
+      <c r="F46" s="47" t="inlineStr">
+        <is>
+          <t>Requisito di agilità: slew di 45° in ≤ 60 s, assestamento escluso (S2). Coppia ≤ 1,0·10⁻³ N·m, picco 1,5°/s, momento ≤ 0,030 N·m·s</t>
+        </is>
+      </c>
+      <c r="G46" s="47" t="inlineStr">
+        <is>
+          <t>S1: 45° in ≤ 120 s (un bersaglio per passaggio); S3: 45° in ≤ 30 s (0,060 N·m·s, 3°/s)</t>
+        </is>
+      </c>
+      <c r="H46" s="47" t="inlineStr">
+        <is>
+          <t>Momento pari a quello della FMC: lo slew non dimensiona le ruote. Con 4 satelliti le zone lontane sono coperte dagli altri; bersagli successivi sullo stesso satellite se distanti ≳ 450 km lungo traccia</t>
+        </is>
+      </c>
+      <c r="I46" s="47" t="inlineStr">
+        <is>
+          <t>Ruote (A5.3 e), DR-08</t>
+        </is>
+      </c>
+      <c r="J46" s="47" t="inlineStr">
+        <is>
+          <t>DR-19, DR-08, MR-05</t>
+        </is>
+      </c>
+      <c r="K46" s="47" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="L46" s="47" t="inlineStr">
+        <is>
+          <t>Approvata</t>
+        </is>
+      </c>
       <c r="M46" s="47" t="n"/>
-      <c r="N46" s="47" t="n"/>
-      <c r="O46" s="47" t="n"/>
+      <c r="N46" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 c) – chat del 24/10/2026</t>
+        </is>
+      </c>
+      <c r="O46" s="47" t="inlineStr">
+        <is>
+          <t>Riguarda solo la parte GNC. Tempo di assestamento dalla simulazione (A5.3 c parte 2)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="26">
-      <c r="A47" s="47" t="n"/>
-      <c r="B47" s="48" t="n"/>
-      <c r="C47" s="47" t="n"/>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="47" t="n"/>
-      <c r="F47" s="47" t="n"/>
-      <c r="G47" s="47" t="n"/>
-      <c r="H47" s="47" t="n"/>
-      <c r="I47" s="47" t="n"/>
-      <c r="J47" s="47" t="n"/>
-      <c r="K47" s="47" t="n"/>
-      <c r="L47" s="47" t="n"/>
+      <c r="A47" s="47" t="inlineStr">
+        <is>
+          <t>D-046</t>
+        </is>
+      </c>
+      <c r="B47" s="48" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C47" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D47" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="E47" s="47" t="inlineStr">
+        <is>
+          <t>GNC</t>
+        </is>
+      </c>
+      <c r="F47" s="47" t="inlineStr">
+        <is>
+          <t>Robustezza del controllo all'inerzia sconosciuta (K3): banda di controllo ~1 rad/s come base, aggiornamento ≥ 10 Hz, anticipo di coppia con l'inerzia stimata in volo al commissioning (entro ~10%); banda riducibile in volo se i pannelli vibrano</t>
+        </is>
+      </c>
+      <c r="G47" s="47" t="inlineStr">
+        <is>
+          <t>K1: solo banda ≥ ~1 rad/s; K2: banda 0,3 rad/s + stima dell'inerzia in volo</t>
+        </is>
+      </c>
+      <c r="H47" s="47" t="inlineStr">
+        <is>
+          <t>Simulazione 1-asse: con banda 1 rad/s 0% di scatti mossi su tutto l'inviluppo (mosso peggiore 2,2–3,7 µrad MEMS, ≤ 0,5 µrad alta qualità, soglia 5,2); con 0,3 rad/s e inerzia vera +65% il 10% degli scatti è mosso e l'APE arriva a 0,22°; con inerzia nota (errore 7%) anche 0,3 rad/s rispetta DR-10. 10 Hz bastano (50 Hz non cambia). Doppia protezione a costo solo software e di commissioning</t>
+        </is>
+      </c>
+      <c r="I47" s="47" t="inlineStr">
+        <is>
+          <t>Software ADCS, procedura di commissioning (stima d'inerzia), A5.3 g), Fase B (3-assi con pannelli)</t>
+        </is>
+      </c>
+      <c r="J47" s="47" t="inlineStr">
+        <is>
+          <t>DR-20, DR-10, DR-15</t>
+        </is>
+      </c>
+      <c r="K47" s="47" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="L47" s="47" t="inlineStr">
+        <is>
+          <t>Approvata</t>
+        </is>
+      </c>
       <c r="M47" s="47" t="n"/>
-      <c r="N47" s="47" t="n"/>
-      <c r="O47" s="47" t="n"/>
+      <c r="N47" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 c) – chat del 24/10/2026; PULSE_ADCS/A5.3 (sim1asse.py, sensibilita.py)</t>
+        </is>
+      </c>
+      <c r="O47" s="47" t="inlineStr">
+        <is>
+          <t>Riguarda solo la parte GNC. Primo esito positivo per D-030 con F2 (conferma in A5.3 g) dopo disturbi e sensori). APE con MEMS 0,067–0,078° vicino al limite: da riprendere in A5.3 f)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="26">
-      <c r="A48" s="47" t="n"/>
-      <c r="B48" s="48" t="n"/>
-      <c r="C48" s="47" t="n"/>
-      <c r="D48" s="47" t="n"/>
-      <c r="E48" s="47" t="n"/>
-      <c r="F48" s="47" t="n"/>
-      <c r="G48" s="47" t="n"/>
-      <c r="H48" s="47" t="n"/>
-      <c r="I48" s="47" t="n"/>
-      <c r="J48" s="47" t="n"/>
-      <c r="K48" s="47" t="n"/>
-      <c r="L48" s="47" t="n"/>
+      <c r="A48" s="47" t="inlineStr">
+        <is>
+          <t>D-047</t>
+        </is>
+      </c>
+      <c r="B48" s="48" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C48" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D48" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="E48" s="47" t="inlineStr">
+        <is>
+          <t>Struttura</t>
+        </is>
+      </c>
+      <c r="F48" s="47" t="inlineStr">
+        <is>
+          <t>Posizione del baricentro (G2): entro 10 mm dalla linea di spinta ed entro 20 mm dal centro di pressione aerodinamico, per tutta la vita (anche con lo iodio consumato). Coppie di progetto: in spinta ~2,3·10⁻⁵ N·m (1,1 mN × 10 mm + aerodinamica + magnetico), in ripresa ~1,4·10⁻⁵ N·m</t>
+        </is>
+      </c>
+      <c r="G48" s="47" t="inlineStr">
+        <is>
+          <t>G1: ≤ 5 mm / ≤ 10 mm (layout e consumo dello iodio troppo vincolati); G3: solo i limiti del deployer DR-14, 45/90 mm (fino a ~1,4·10⁻⁴ N·m, ruote sature in spinta)</t>
+        </is>
+      </c>
+      <c r="H48" s="47" t="inlineStr">
+        <is>
+          <t>La spinta disallineata è la coppia dominante, come in EarthNext. Con 90 mm il momento da scaricare in 4,2 h di spinta è 1,50 N·m·s, oltre i magnetorquer di classe EarthNext (2,6 A·m², 6,8·10⁻⁵–1,4·10⁻⁴ N·m di picco); con 10 mm 0,17 N·m·s, scaricabile di continuo. Ordine di grandezza coerente con EarthNext Tab. 4. Densità dimensionante 4,6·10⁻¹¹ kg/m³ (MSIS, F10.7 181, Ap 50); la simulazione F2 non cambia mosso con disturbi fino a 10⁻⁴ N·m</t>
+        </is>
+      </c>
+      <c r="I48" s="47" t="inlineStr">
+        <is>
+          <t>Layout e bilanciamento (A5.7), posizione del telescopio (Giuseppe) e della REGULUS, magnetorquer (A5.3 e), DR-14</t>
+        </is>
+      </c>
+      <c r="J48" s="47" t="inlineStr">
+        <is>
+          <t>DR-21, DR-14</t>
+        </is>
+      </c>
+      <c r="K48" s="47" t="inlineStr">
+        <is>
+          <t>R-26, R-06</t>
+        </is>
+      </c>
+      <c r="L48" s="47" t="inlineStr">
+        <is>
+          <t>Proposta</t>
+        </is>
+      </c>
       <c r="M48" s="47" t="n"/>
-      <c r="N48" s="47" t="n"/>
-      <c r="O48" s="47" t="n"/>
+      <c r="N48" s="47" t="inlineStr">
+        <is>
+          <t>A5.3 d) – chat del 24/10/2026; PULSE_ADCS/A5.3/disturbi.py</t>
+        </is>
+      </c>
+      <c r="O48" s="47" t="inlineStr">
+        <is>
+          <t>Proposta: vincola il layout in comune e la posizione del telescopio. DR-14 resta il limite del deployer; DR-21 è il requisito di progetto ADCS, molto più stretto. Valori TBC</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="26">
       <c r="A49" s="47" t="n"/>
@@ -5225,7 +5495,7 @@
       </c>
       <c r="I21" s="47" t="inlineStr">
         <is>
-          <t>A5.3 a): scelta C (D-040, Proposta). Prima: ≤ 0,0002°/s senza correzione oppure ~0,001°/s con riallineamento a terra (scartato: contraddice D-007/MR-10). Ritardo tra le bande ~0,79 s (stima)</t>
+          <t>A5.3 a): scelta C (D-040, Proposta). Prima: ≤ 0,0002°/s senza correzione oppure ~0,001°/s con riallineamento a terra (scartato: contraddice D-007/MR-10). Ritardo tra le bande ~0,79 s (stima). A5.3 c): la rotazione terrestre fa scorrere il terreno di traverso di 2,4–2,9° (~250–290 m in 0,79 s): spostamento noto, da compensare (yaw steering o correzione a bordo) in A5.3 g)</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5773,7 @@
       </c>
       <c r="I27" s="47" t="inlineStr">
         <is>
-          <t>Esclusi puntamento e assestamento</t>
+          <t>Esclusi puntamento e assestamento. A5.3 c): con il profilo F2 (D-044) l'inseguimento dura tutta la finestra (47,7 s a 30°), ben oltre 0,36 s</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5914,7 @@
       </c>
       <c r="I30" s="47" t="inlineStr">
         <is>
-          <t>Valori del manuale EXOpod Nova; telescopio (Giuseppe) e propulsione ~6 kg (Giuliano) sono le masse da bilanciare</t>
+          <t>Valori del manuale EXOpod Nova; telescopio (Giuseppe) e propulsione ~6 kg (Giuliano) sono le masse da bilanciare. A5.3 d): per l'ADCS vale il requisito più stretto DR-21 (D-047)</t>
         </is>
       </c>
     </row>
@@ -5837,37 +6107,145 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="26">
-      <c r="A35" s="47" t="n"/>
-      <c r="B35" s="47" t="n"/>
-      <c r="C35" s="47" t="n"/>
-      <c r="D35" s="47" t="n"/>
-      <c r="E35" s="47" t="n"/>
-      <c r="F35" s="47" t="n"/>
-      <c r="G35" s="47" t="n"/>
-      <c r="H35" s="47" t="n"/>
-      <c r="I35" s="47" t="n"/>
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>DR-19</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>Derivato</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>Il satellite deve ruotare di 45° (slew) per puntare un nuovo bersaglio entro il tempo stabilito, assestamento escluso.</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>45° in ≤ 60 s</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>Analisi + simulazione GNC</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="G35" s="47" t="inlineStr">
+        <is>
+          <t>D-045 (A5)</t>
+        </is>
+      </c>
+      <c r="H35" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="I35" s="47" t="inlineStr">
+        <is>
+          <t>Coppia ≤ 1,0·10⁻³ N·m, picco 1,5°/s, momento ≤ 0,030 N·m·s con I = 1,14 kg·m²</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="26">
-      <c r="A36" s="47" t="n"/>
-      <c r="B36" s="47" t="n"/>
-      <c r="C36" s="47" t="n"/>
-      <c r="D36" s="47" t="n"/>
-      <c r="E36" s="47" t="n"/>
-      <c r="F36" s="47" t="n"/>
-      <c r="G36" s="47" t="n"/>
-      <c r="H36" s="47" t="n"/>
-      <c r="I36" s="47" t="n"/>
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>DR-20</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>Derivato</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Il controllo d'assetto deve inseguire la linea di vista nonostante l'incertezza d'inerzia, con anticipo di coppia basato sull'inerzia stimata in volo.</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>banda ~1 rad/s; aggiornamento ≥ 10 Hz; inerzia stimata entro ~10%</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="inlineStr">
+        <is>
+          <t>Simulazione GNC (1-asse in A, 3-assi in B), test in commissioning</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="G36" s="47" t="inlineStr">
+        <is>
+          <t>D-046 (A5)</t>
+        </is>
+      </c>
+      <c r="H36" s="47" t="inlineStr">
+        <is>
+          <t>Giuliano</t>
+        </is>
+      </c>
+      <c r="I36" s="47" t="inlineStr">
+        <is>
+          <t>Errore d'inerzia del 7% verificato con banda 0,3 rad/s; banda da ricontrollare in Fase B con i modi flessibili dei pannelli</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="26">
-      <c r="A37" s="47" t="n"/>
-      <c r="B37" s="47" t="n"/>
-      <c r="C37" s="47" t="n"/>
-      <c r="D37" s="47" t="n"/>
-      <c r="E37" s="47" t="n"/>
-      <c r="F37" s="47" t="n"/>
-      <c r="G37" s="47" t="n"/>
-      <c r="H37" s="47" t="n"/>
-      <c r="I37" s="47" t="n"/>
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>DR-21</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="inlineStr">
+        <is>
+          <t>Derivato</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Il baricentro del satellite deve restare vicino alla linea di spinta e al centro di pressione aerodinamico per tutta la vita operativa, anche con lo iodio consumato.</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>≤ 10 mm dalla linea di spinta; ≤ 20 mm dal centro di pressione</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>Analisi (modello di massa), poi misura e bilanciamento</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="G37" s="47" t="inlineStr">
+        <is>
+          <t>D-047 (A5)</t>
+        </is>
+      </c>
+      <c r="H37" s="47" t="inlineStr">
+        <is>
+          <t>Entrambi</t>
+        </is>
+      </c>
+      <c r="I37" s="47" t="inlineStr">
+        <is>
+          <t>Più stretto di DR-14 (limite del deployer). Coppia da spinta 1,1·10⁻⁵ N·m a 1,1 mN; aerodinamica 6,9·10⁻⁶ N·m alla densità dimensionante. Verifica in A5.7</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="26">
       <c r="A38" s="47" t="n"/>
@@ -6445,7 +6823,7 @@
       </c>
       <c r="M7" s="47" t="inlineStr">
         <is>
-          <t>A3: deriva &lt; 0,015°/s per scatto, inseguimento 0,36 s (DR-10, DR-11)</t>
+          <t>A3: deriva &lt; 0,015°/s per scatto, inseguimento 0,36 s (DR-10, DR-11). A5.3 c): simulazione 1-asse, F2 rispetta DR-10 con banda 1 rad/s (D-044, D-046); F1 a 7 mN·m satura la ruota di prova con inerzia massima. A5.3 d): disturbi fino a 10⁻⁴ N·m non cambiano il mosso; il rischio vero è la saturazione in spinta (R-26)</t>
         </is>
       </c>
     </row>
@@ -7560,22 +7938,62 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="26">
-      <c r="A27" s="47" t="n"/>
-      <c r="B27" s="47" t="n"/>
-      <c r="C27" s="47" t="n"/>
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>R-26</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="inlineStr">
+        <is>
+          <t>Baricentro fuori dai limiti di DR-21 (layout, tolleranze, spostamento con il consumo dello iodio)</t>
+        </is>
+      </c>
+      <c r="C27" s="47" t="inlineStr">
+        <is>
+          <t>Coppia da spinta e aerodinamica più alte: ruote sature durante la spinta, spinte interrotte, mantenimento della quota più difficile</t>
+        </is>
+      </c>
       <c r="D27" s="47" t="n"/>
-      <c r="E27" s="47" t="n"/>
+      <c r="E27" s="47" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
       <c r="F27" s="50">
         <f>IF(OR(D27="",E27=""),"",MATCH(D27,{"Bassa","Media","Alta"},0)*MATCH(E27,{"Bassa","Media","Alta"},0))</f>
         <v/>
       </c>
-      <c r="G27" s="47" t="n"/>
-      <c r="H27" s="47" t="n"/>
+      <c r="G27" s="47" t="inlineStr">
+        <is>
+          <t>Bilanciamento nel layout (A5.7), serbatoio vicino al baricentro, zavorra, misura del baricentro a terra; magnetorquer con margine (A5.3 e); in volo spinta a intervalli con desaturazioni</t>
+        </is>
+      </c>
+      <c r="H27" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
       <c r="I27" s="47" t="n"/>
-      <c r="J27" s="47" t="n"/>
-      <c r="K27" s="47" t="n"/>
-      <c r="L27" s="47" t="n"/>
-      <c r="M27" s="47" t="n"/>
+      <c r="J27" s="47" t="inlineStr">
+        <is>
+          <t>Entrambi</t>
+        </is>
+      </c>
+      <c r="K27" s="47" t="inlineStr">
+        <is>
+          <t>Aperto</t>
+        </is>
+      </c>
+      <c r="L27" s="47" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="M27" s="47" t="inlineStr">
+        <is>
+          <t>Nato in A5.3 d) (D-047). Con il baricentro al limite del deployer (90 mm) la coppia di spinta è ~10⁻⁴ N·m. Probabilità da valutare in A6</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="26">
       <c r="A28" s="47" t="n"/>

</xml_diff>